<commit_message>
fig14 Excel: unbroken lines (dropped points removed), y-axis fitted to data, larger chart, legend at bottom
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig14_lines.xlsx
+++ b/figs/data/fig14_lines.xlsx
@@ -174,12 +174,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'OLTP→Varmail'!$A$2:$A$62</f>
+              <f>'OLTP→Varmail'!$A$2:$A$61</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'OLTP→Varmail'!$B$2:$B$62</f>
+              <f>'OLTP→Varmail'!$B$2:$B$61</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -210,12 +210,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'OLTP→Varmail'!$C$2:$C$62</f>
+              <f>'OLTP→Varmail'!$C$2:$C$61</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'OLTP→Varmail'!$D$2:$D$62</f>
+              <f>'OLTP→Varmail'!$D$2:$D$61</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -246,12 +246,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'OLTP→Varmail'!$E$2:$E$62</f>
+              <f>'OLTP→Varmail'!$E$2:$E$61</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'OLTP→Varmail'!$F$2:$F$62</f>
+              <f>'OLTP→Varmail'!$F$2:$F$61</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -282,12 +282,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'OLTP→Varmail'!$G$2:$G$62</f>
+              <f>'OLTP→Varmail'!$G$2:$G$61</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'OLTP→Varmail'!$H$2:$H$62</f>
+              <f>'OLTP→Varmail'!$H$2:$H$61</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -299,6 +299,8 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="31"/>
+          <min val="0"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -318,14 +320,18 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
+        <majorUnit val="5"/>
       </valAx>
       <valAx>
         <axId val="20"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="2.5"/>
+          <min val="1.12"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -345,13 +351,14 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0.00" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -531,6 +538,8 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="45"/>
+          <min val="0"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -550,14 +559,18 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
+        <majorUnit val="5"/>
       </valAx>
       <valAx>
         <axId val="20"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="4.41"/>
+          <min val="1.45"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -577,13 +590,14 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0.00" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -638,12 +652,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'YCSB-A→YCSB-B'!$A$2:$A$40</f>
+              <f>'YCSB-A→YCSB-B'!$A$2:$A$39</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'YCSB-A→YCSB-B'!$B$2:$B$40</f>
+              <f>'YCSB-A→YCSB-B'!$B$2:$B$39</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -674,12 +688,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'YCSB-A→YCSB-B'!$C$2:$C$40</f>
+              <f>'YCSB-A→YCSB-B'!$C$2:$C$39</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'YCSB-A→YCSB-B'!$D$2:$D$40</f>
+              <f>'YCSB-A→YCSB-B'!$D$2:$D$39</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -710,12 +724,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'YCSB-A→YCSB-B'!$E$2:$E$40</f>
+              <f>'YCSB-A→YCSB-B'!$E$2:$E$39</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'YCSB-A→YCSB-B'!$F$2:$F$40</f>
+              <f>'YCSB-A→YCSB-B'!$F$2:$F$39</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -746,12 +760,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'YCSB-A→YCSB-B'!$G$2:$G$40</f>
+              <f>'YCSB-A→YCSB-B'!$G$2:$G$39</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'YCSB-A→YCSB-B'!$H$2:$H$40</f>
+              <f>'YCSB-A→YCSB-B'!$H$2:$H$39</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -763,6 +777,8 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="20"/>
+          <min val="0"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -782,14 +798,18 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
+        <majorUnit val="5"/>
       </valAx>
       <valAx>
         <axId val="20"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="1.7"/>
+          <min val="1.25"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -809,13 +829,14 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0.00" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -995,6 +1016,8 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="20"/>
+          <min val="0"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -1014,14 +1037,18 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="20"/>
+        <majorUnit val="5"/>
       </valAx>
       <valAx>
         <axId val="20"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="2.04"/>
+          <min val="0.92"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -1041,13 +1068,14 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0.00" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
     <legend>
-      <legendPos val="r"/>
+      <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
@@ -1064,7 +1092,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="3960000"/>
+    <ext cx="10800000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1091,7 +1119,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="3960000"/>
+    <ext cx="10800000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1118,7 +1146,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="3960000"/>
+    <ext cx="10800000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1145,7 +1173,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="3960000"/>
+    <ext cx="10800000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1452,8 +1480,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2050,7 +2081,10 @@
         <v>1.2255</v>
       </c>
       <c r="C22" t="n">
-        <v>10.53</v>
+        <v>11.08</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1.2529</v>
       </c>
       <c r="E22" t="n">
         <v>10.52</v>
@@ -2073,10 +2107,10 @@
         <v>1.2259</v>
       </c>
       <c r="C23" t="n">
-        <v>11.08</v>
+        <v>11.58</v>
       </c>
       <c r="D23" t="n">
-        <v>1.2529</v>
+        <v>1.2528</v>
       </c>
       <c r="E23" t="n">
         <v>11.02</v>
@@ -2099,10 +2133,10 @@
         <v>1.226</v>
       </c>
       <c r="C24" t="n">
-        <v>11.58</v>
+        <v>12.1</v>
       </c>
       <c r="D24" t="n">
-        <v>1.2528</v>
+        <v>1.2529</v>
       </c>
       <c r="E24" t="n">
         <v>11.52</v>
@@ -2125,10 +2159,10 @@
         <v>1.2334</v>
       </c>
       <c r="C25" t="n">
-        <v>12.1</v>
+        <v>12.6</v>
       </c>
       <c r="D25" t="n">
-        <v>1.2529</v>
+        <v>1.2532</v>
       </c>
       <c r="E25" t="n">
         <v>12.02</v>
@@ -2151,10 +2185,10 @@
         <v>1.2232</v>
       </c>
       <c r="C26" t="n">
-        <v>12.6</v>
+        <v>13.1</v>
       </c>
       <c r="D26" t="n">
-        <v>1.2532</v>
+        <v>1.2523</v>
       </c>
       <c r="E26" t="n">
         <v>12.52</v>
@@ -2177,10 +2211,10 @@
         <v>1.2265</v>
       </c>
       <c r="C27" t="n">
-        <v>13.1</v>
+        <v>13.6</v>
       </c>
       <c r="D27" t="n">
-        <v>1.2523</v>
+        <v>1.2525</v>
       </c>
       <c r="E27" t="n">
         <v>13.02</v>
@@ -2203,10 +2237,10 @@
         <v>1.2197</v>
       </c>
       <c r="C28" t="n">
-        <v>13.6</v>
+        <v>14.1</v>
       </c>
       <c r="D28" t="n">
-        <v>1.2525</v>
+        <v>1.2526</v>
       </c>
       <c r="E28" t="n">
         <v>13.52</v>
@@ -2229,10 +2263,10 @@
         <v>1.2197</v>
       </c>
       <c r="C29" t="n">
-        <v>14.1</v>
+        <v>14.6</v>
       </c>
       <c r="D29" t="n">
-        <v>1.2526</v>
+        <v>1.2538</v>
       </c>
       <c r="E29" t="n">
         <v>14.02</v>
@@ -2255,10 +2289,10 @@
         <v>1.2198</v>
       </c>
       <c r="C30" t="n">
-        <v>14.6</v>
+        <v>15.1</v>
       </c>
       <c r="D30" t="n">
-        <v>1.2538</v>
+        <v>1.2515</v>
       </c>
       <c r="E30" t="n">
         <v>14.52</v>
@@ -2281,10 +2315,10 @@
         <v>1.2199</v>
       </c>
       <c r="C31" t="n">
-        <v>15.1</v>
+        <v>15.6</v>
       </c>
       <c r="D31" t="n">
-        <v>1.2515</v>
+        <v>1.6821</v>
       </c>
       <c r="E31" t="n">
         <v>15.02</v>
@@ -2301,13 +2335,16 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>15.53</v>
+        <v>16.03</v>
+      </c>
+      <c r="B32" t="n">
+        <v>1.5036</v>
       </c>
       <c r="C32" t="n">
-        <v>15.6</v>
+        <v>16.1</v>
       </c>
       <c r="D32" t="n">
-        <v>1.6821</v>
+        <v>1.9809</v>
       </c>
       <c r="E32" t="n">
         <v>15.52</v>
@@ -2324,16 +2361,16 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>16.03</v>
+        <v>16.53</v>
       </c>
       <c r="B33" t="n">
-        <v>1.5036</v>
+        <v>1.9627</v>
       </c>
       <c r="C33" t="n">
-        <v>16.1</v>
+        <v>16.6</v>
       </c>
       <c r="D33" t="n">
-        <v>1.9809</v>
+        <v>2.0074</v>
       </c>
       <c r="E33" t="n">
         <v>16.02</v>
@@ -2350,16 +2387,16 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>16.53</v>
+        <v>17.03</v>
       </c>
       <c r="B34" t="n">
-        <v>1.9627</v>
+        <v>1.9591</v>
       </c>
       <c r="C34" t="n">
-        <v>16.6</v>
+        <v>17.1</v>
       </c>
       <c r="D34" t="n">
-        <v>2.0074</v>
+        <v>2.011</v>
       </c>
       <c r="E34" t="n">
         <v>16.52</v>
@@ -2376,16 +2413,16 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>17.03</v>
+        <v>17.53</v>
       </c>
       <c r="B35" t="n">
-        <v>1.9591</v>
+        <v>1.9602</v>
       </c>
       <c r="C35" t="n">
-        <v>17.1</v>
+        <v>17.6</v>
       </c>
       <c r="D35" t="n">
-        <v>2.011</v>
+        <v>2.0183</v>
       </c>
       <c r="E35" t="n">
         <v>17.02</v>
@@ -2402,16 +2439,16 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>17.53</v>
+        <v>18.03</v>
       </c>
       <c r="B36" t="n">
-        <v>1.9602</v>
+        <v>1.9649</v>
       </c>
       <c r="C36" t="n">
-        <v>17.6</v>
+        <v>18.1</v>
       </c>
       <c r="D36" t="n">
-        <v>2.0183</v>
+        <v>2.0225</v>
       </c>
       <c r="E36" t="n">
         <v>17.52</v>
@@ -2428,16 +2465,16 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>18.03</v>
+        <v>18.53</v>
       </c>
       <c r="B37" t="n">
-        <v>1.9649</v>
+        <v>1.9705</v>
       </c>
       <c r="C37" t="n">
-        <v>18.1</v>
+        <v>18.6</v>
       </c>
       <c r="D37" t="n">
-        <v>2.0225</v>
+        <v>2.0224</v>
       </c>
       <c r="E37" t="n">
         <v>18.02</v>
@@ -2454,16 +2491,16 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>18.53</v>
+        <v>19.03</v>
       </c>
       <c r="B38" t="n">
-        <v>1.9705</v>
+        <v>1.9668</v>
       </c>
       <c r="C38" t="n">
-        <v>18.6</v>
+        <v>19.1</v>
       </c>
       <c r="D38" t="n">
-        <v>2.0224</v>
+        <v>2.0231</v>
       </c>
       <c r="E38" t="n">
         <v>18.52</v>
@@ -2480,16 +2517,16 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>19.03</v>
+        <v>19.53</v>
       </c>
       <c r="B39" t="n">
-        <v>1.9668</v>
+        <v>1.9673</v>
       </c>
       <c r="C39" t="n">
-        <v>19.1</v>
+        <v>19.6</v>
       </c>
       <c r="D39" t="n">
-        <v>2.0231</v>
+        <v>2.0256</v>
       </c>
       <c r="E39" t="n">
         <v>19.02</v>
@@ -2506,16 +2543,16 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>19.53</v>
+        <v>20.03</v>
       </c>
       <c r="B40" t="n">
-        <v>1.9673</v>
+        <v>1.9674</v>
       </c>
       <c r="C40" t="n">
-        <v>19.6</v>
+        <v>20.1</v>
       </c>
       <c r="D40" t="n">
-        <v>2.0256</v>
+        <v>2.0252</v>
       </c>
       <c r="E40" t="n">
         <v>19.52</v>
@@ -2532,16 +2569,16 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>20.03</v>
+        <v>20.53</v>
       </c>
       <c r="B41" t="n">
-        <v>1.9674</v>
+        <v>1.9679</v>
       </c>
       <c r="C41" t="n">
-        <v>20.1</v>
+        <v>20.6</v>
       </c>
       <c r="D41" t="n">
-        <v>2.0252</v>
+        <v>2.0256</v>
       </c>
       <c r="E41" t="n">
         <v>20.02</v>
@@ -2558,16 +2595,16 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>20.53</v>
+        <v>21.03</v>
       </c>
       <c r="B42" t="n">
-        <v>1.9679</v>
+        <v>1.9695</v>
       </c>
       <c r="C42" t="n">
-        <v>20.6</v>
+        <v>21.1</v>
       </c>
       <c r="D42" t="n">
-        <v>2.0256</v>
+        <v>2.0234</v>
       </c>
       <c r="E42" t="n">
         <v>20.52</v>
@@ -2584,16 +2621,16 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>21.03</v>
+        <v>21.53</v>
       </c>
       <c r="B43" t="n">
-        <v>1.9695</v>
+        <v>1.965</v>
       </c>
       <c r="C43" t="n">
-        <v>21.1</v>
+        <v>21.6</v>
       </c>
       <c r="D43" t="n">
-        <v>2.0234</v>
+        <v>2.0273</v>
       </c>
       <c r="E43" t="n">
         <v>21.02</v>
@@ -2610,16 +2647,16 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>21.53</v>
+        <v>22.03</v>
       </c>
       <c r="B44" t="n">
-        <v>1.965</v>
+        <v>1.9669</v>
       </c>
       <c r="C44" t="n">
-        <v>21.6</v>
+        <v>22.1</v>
       </c>
       <c r="D44" t="n">
-        <v>2.0273</v>
+        <v>2.0238</v>
       </c>
       <c r="E44" t="n">
         <v>21.52</v>
@@ -2636,16 +2673,16 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>22.03</v>
+        <v>22.53</v>
       </c>
       <c r="B45" t="n">
-        <v>1.9669</v>
+        <v>1.9661</v>
       </c>
       <c r="C45" t="n">
-        <v>22.1</v>
+        <v>22.6</v>
       </c>
       <c r="D45" t="n">
-        <v>2.0238</v>
+        <v>2.0249</v>
       </c>
       <c r="E45" t="n">
         <v>22.02</v>
@@ -2662,16 +2699,16 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>22.53</v>
+        <v>23.03</v>
       </c>
       <c r="B46" t="n">
-        <v>1.9661</v>
+        <v>1.9686</v>
       </c>
       <c r="C46" t="n">
-        <v>22.6</v>
+        <v>23.1</v>
       </c>
       <c r="D46" t="n">
-        <v>2.0249</v>
+        <v>2.0285</v>
       </c>
       <c r="E46" t="n">
         <v>22.52</v>
@@ -2688,16 +2725,16 @@
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>23.03</v>
+        <v>23.53</v>
       </c>
       <c r="B47" t="n">
-        <v>1.9686</v>
+        <v>1.9683</v>
       </c>
       <c r="C47" t="n">
-        <v>23.1</v>
+        <v>23.6</v>
       </c>
       <c r="D47" t="n">
-        <v>2.0285</v>
+        <v>2.025</v>
       </c>
       <c r="E47" t="n">
         <v>23.02</v>
@@ -2714,16 +2751,16 @@
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>23.53</v>
+        <v>24.03</v>
       </c>
       <c r="B48" t="n">
-        <v>1.9683</v>
+        <v>1.969</v>
       </c>
       <c r="C48" t="n">
-        <v>23.6</v>
+        <v>24.1</v>
       </c>
       <c r="D48" t="n">
-        <v>2.025</v>
+        <v>2.0243</v>
       </c>
       <c r="E48" t="n">
         <v>23.52</v>
@@ -2740,16 +2777,16 @@
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>24.03</v>
+        <v>24.53</v>
       </c>
       <c r="B49" t="n">
-        <v>1.969</v>
+        <v>1.9731</v>
       </c>
       <c r="C49" t="n">
-        <v>24.1</v>
+        <v>24.6</v>
       </c>
       <c r="D49" t="n">
-        <v>2.0243</v>
+        <v>2.0255</v>
       </c>
       <c r="E49" t="n">
         <v>24.02</v>
@@ -2766,16 +2803,16 @@
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>24.53</v>
+        <v>25.03</v>
       </c>
       <c r="B50" t="n">
-        <v>1.9731</v>
+        <v>1.967</v>
       </c>
       <c r="C50" t="n">
-        <v>24.6</v>
+        <v>25.1</v>
       </c>
       <c r="D50" t="n">
-        <v>2.0255</v>
+        <v>2.0265</v>
       </c>
       <c r="E50" t="n">
         <v>24.52</v>
@@ -2792,16 +2829,16 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>25.03</v>
+        <v>25.53</v>
       </c>
       <c r="B51" t="n">
-        <v>1.967</v>
+        <v>1.9673</v>
       </c>
       <c r="C51" t="n">
-        <v>25.1</v>
+        <v>25.6</v>
       </c>
       <c r="D51" t="n">
-        <v>2.0265</v>
+        <v>2.0251</v>
       </c>
       <c r="E51" t="n">
         <v>25.02</v>
@@ -2818,16 +2855,16 @@
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>25.53</v>
+        <v>26.03</v>
       </c>
       <c r="B52" t="n">
-        <v>1.9673</v>
+        <v>1.9619</v>
       </c>
       <c r="C52" t="n">
-        <v>25.6</v>
+        <v>26.1</v>
       </c>
       <c r="D52" t="n">
-        <v>2.0251</v>
+        <v>2.0261</v>
       </c>
       <c r="E52" t="n">
         <v>25.52</v>
@@ -2844,16 +2881,16 @@
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>26.03</v>
+        <v>26.53</v>
       </c>
       <c r="B53" t="n">
-        <v>1.9619</v>
+        <v>1.9612</v>
       </c>
       <c r="C53" t="n">
-        <v>26.1</v>
+        <v>26.6</v>
       </c>
       <c r="D53" t="n">
-        <v>2.0261</v>
+        <v>2.0244</v>
       </c>
       <c r="E53" t="n">
         <v>26.02</v>
@@ -2870,16 +2907,16 @@
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>26.53</v>
+        <v>27.03</v>
       </c>
       <c r="B54" t="n">
-        <v>1.9612</v>
+        <v>1.9649</v>
       </c>
       <c r="C54" t="n">
-        <v>26.6</v>
+        <v>27.1</v>
       </c>
       <c r="D54" t="n">
-        <v>2.0244</v>
+        <v>2.0275</v>
       </c>
       <c r="E54" t="n">
         <v>26.52</v>
@@ -2896,16 +2933,16 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>27.03</v>
+        <v>27.53</v>
       </c>
       <c r="B55" t="n">
-        <v>1.9649</v>
+        <v>1.9664</v>
       </c>
       <c r="C55" t="n">
-        <v>27.1</v>
+        <v>27.6</v>
       </c>
       <c r="D55" t="n">
-        <v>2.0275</v>
+        <v>2.0265</v>
       </c>
       <c r="E55" t="n">
         <v>27.02</v>
@@ -2922,16 +2959,16 @@
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>27.53</v>
+        <v>28.03</v>
       </c>
       <c r="B56" t="n">
-        <v>1.9664</v>
+        <v>1.9675</v>
       </c>
       <c r="C56" t="n">
-        <v>27.6</v>
+        <v>28.1</v>
       </c>
       <c r="D56" t="n">
-        <v>2.0265</v>
+        <v>2.026</v>
       </c>
       <c r="E56" t="n">
         <v>27.52</v>
@@ -2948,16 +2985,16 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>28.03</v>
+        <v>28.53</v>
       </c>
       <c r="B57" t="n">
-        <v>1.9675</v>
+        <v>1.9603</v>
       </c>
       <c r="C57" t="n">
-        <v>28.1</v>
+        <v>28.6</v>
       </c>
       <c r="D57" t="n">
-        <v>2.026</v>
+        <v>2.0228</v>
       </c>
       <c r="E57" t="n">
         <v>28.02</v>
@@ -2974,16 +3011,16 @@
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>28.53</v>
+        <v>29.03</v>
       </c>
       <c r="B58" t="n">
-        <v>1.9603</v>
+        <v>1.9619</v>
       </c>
       <c r="C58" t="n">
-        <v>28.6</v>
+        <v>29.1</v>
       </c>
       <c r="D58" t="n">
-        <v>2.0228</v>
+        <v>2.0245</v>
       </c>
       <c r="E58" t="n">
         <v>28.52</v>
@@ -3000,16 +3037,16 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>29.03</v>
+        <v>29.53</v>
       </c>
       <c r="B59" t="n">
-        <v>1.9619</v>
+        <v>1.9601</v>
       </c>
       <c r="C59" t="n">
-        <v>29.1</v>
+        <v>29.6</v>
       </c>
       <c r="D59" t="n">
-        <v>2.0245</v>
+        <v>2.024</v>
       </c>
       <c r="E59" t="n">
         <v>29.02</v>
@@ -3026,16 +3063,16 @@
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>29.53</v>
+        <v>30.03</v>
       </c>
       <c r="B60" t="n">
-        <v>1.9601</v>
+        <v>1.9615</v>
       </c>
       <c r="C60" t="n">
-        <v>29.6</v>
+        <v>30.1</v>
       </c>
       <c r="D60" t="n">
-        <v>2.024</v>
+        <v>2.026</v>
       </c>
       <c r="E60" t="n">
         <v>29.52</v>
@@ -3052,30 +3089,16 @@
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>30.03</v>
+        <v>30.53</v>
       </c>
       <c r="B61" t="n">
-        <v>1.9615</v>
-      </c>
-      <c r="C61" t="n">
-        <v>30.1</v>
-      </c>
-      <c r="D61" t="n">
-        <v>2.026</v>
+        <v>1.9625</v>
       </c>
       <c r="E61" t="n">
         <v>30.02</v>
       </c>
       <c r="F61" t="n">
         <v>2.0966</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n">
-        <v>30.53</v>
-      </c>
-      <c r="B62" t="n">
-        <v>1.9625</v>
       </c>
     </row>
   </sheetData>
@@ -3092,6 +3115,9 @@
   </sheetPr>
   <dimension ref="A1:J90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -5486,8 +5512,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6364,7 +6393,10 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>16.27</v>
+        <v>16.78</v>
+      </c>
+      <c r="B33" t="n">
+        <v>1.2849</v>
       </c>
       <c r="C33" t="n">
         <v>16.28</v>
@@ -6373,7 +6405,10 @@
         <v>1.408</v>
       </c>
       <c r="E33" t="n">
-        <v>16.38</v>
+        <v>16.88</v>
+      </c>
+      <c r="F33" t="n">
+        <v>1.3354</v>
       </c>
       <c r="G33" t="n">
         <v>16.32</v>
@@ -6384,156 +6419,133 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>16.78</v>
+        <v>17.28</v>
       </c>
       <c r="B34" t="n">
-        <v>1.2849</v>
+        <v>1.3554</v>
       </c>
       <c r="C34" t="n">
-        <v>16.87</v>
+        <v>17.37</v>
+      </c>
+      <c r="D34" t="n">
+        <v>1.3422</v>
       </c>
       <c r="E34" t="n">
-        <v>16.88</v>
+        <v>17.4</v>
       </c>
       <c r="F34" t="n">
-        <v>1.3354</v>
+        <v>1.3486</v>
       </c>
       <c r="G34" t="n">
-        <v>16.97</v>
+        <v>17.47</v>
+      </c>
+      <c r="H34" t="n">
+        <v>1.4821</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>17.28</v>
+        <v>17.78</v>
       </c>
       <c r="B35" t="n">
-        <v>1.3554</v>
+        <v>1.405</v>
       </c>
       <c r="C35" t="n">
-        <v>17.37</v>
+        <v>17.88</v>
       </c>
       <c r="D35" t="n">
-        <v>1.3422</v>
+        <v>1.4323</v>
       </c>
       <c r="E35" t="n">
-        <v>17.4</v>
+        <v>17.9</v>
       </c>
       <c r="F35" t="n">
-        <v>1.3486</v>
+        <v>1.4496</v>
       </c>
       <c r="G35" t="n">
-        <v>17.47</v>
+        <v>17.98</v>
       </c>
       <c r="H35" t="n">
-        <v>1.4821</v>
+        <v>1.4075</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>17.78</v>
+        <v>18.3</v>
       </c>
       <c r="B36" t="n">
-        <v>1.405</v>
+        <v>1.3827</v>
       </c>
       <c r="C36" t="n">
-        <v>17.88</v>
+        <v>18.42</v>
       </c>
       <c r="D36" t="n">
-        <v>1.4323</v>
+        <v>1.4652</v>
       </c>
       <c r="E36" t="n">
-        <v>17.9</v>
+        <v>18.42</v>
       </c>
       <c r="F36" t="n">
-        <v>1.4496</v>
+        <v>1.4421</v>
       </c>
       <c r="G36" t="n">
-        <v>17.98</v>
+        <v>18.68</v>
       </c>
       <c r="H36" t="n">
-        <v>1.4075</v>
+        <v>1.4467</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>18.3</v>
+        <v>18.8</v>
       </c>
       <c r="B37" t="n">
-        <v>1.3827</v>
+        <v>1.3279</v>
       </c>
       <c r="C37" t="n">
-        <v>18.42</v>
+        <v>18.92</v>
       </c>
       <c r="D37" t="n">
-        <v>1.4652</v>
+        <v>1.4721</v>
       </c>
       <c r="E37" t="n">
-        <v>18.42</v>
+        <v>18.93</v>
       </c>
       <c r="F37" t="n">
-        <v>1.4421</v>
+        <v>1.4474</v>
       </c>
       <c r="G37" t="n">
-        <v>18.68</v>
+        <v>19.27</v>
       </c>
       <c r="H37" t="n">
-        <v>1.4467</v>
+        <v>1.4759</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="B38" t="n">
-        <v>1.3279</v>
-      </c>
       <c r="C38" t="n">
-        <v>18.92</v>
+        <v>19.42</v>
       </c>
       <c r="D38" t="n">
-        <v>1.4721</v>
+        <v>1.4644</v>
       </c>
       <c r="E38" t="n">
-        <v>18.93</v>
+        <v>19.45</v>
       </c>
       <c r="F38" t="n">
-        <v>1.4474</v>
+        <v>1.392</v>
       </c>
       <c r="G38" t="n">
-        <v>19.27</v>
+        <v>19.78</v>
       </c>
       <c r="H38" t="n">
-        <v>1.4759</v>
+        <v>1.4659</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="n">
-        <v>19.33</v>
-      </c>
       <c r="C39" t="n">
-        <v>19.42</v>
+        <v>19.97</v>
       </c>
       <c r="D39" t="n">
-        <v>1.4644</v>
-      </c>
-      <c r="E39" t="n">
-        <v>19.45</v>
-      </c>
-      <c r="F39" t="n">
-        <v>1.392</v>
-      </c>
-      <c r="G39" t="n">
-        <v>19.78</v>
-      </c>
-      <c r="H39" t="n">
-        <v>1.4659</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="C40" t="n">
-        <v>19.97</v>
-      </c>
-      <c r="D40" t="n">
         <v>1.4592</v>
       </c>
     </row>
@@ -6551,6 +6563,9 @@
   </sheetPr>
   <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="10" max="10"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -6694,7 +6709,10 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2.03</v>
+        <v>3.55</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1.3455</v>
       </c>
       <c r="C5" t="n">
         <v>2.03</v>
@@ -6722,7 +6740,10 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2.53</v>
+        <v>4.05</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1.2272</v>
       </c>
       <c r="C6" t="n">
         <v>2.53</v>
@@ -6737,12 +6758,18 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>2.53</v>
+        <v>3.05</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>3.05</v>
+        <v>4.55</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1.1073</v>
       </c>
       <c r="C7" t="n">
         <v>3.05</v>
@@ -6757,18 +6784,18 @@
         <v>1.0003</v>
       </c>
       <c r="G7" t="n">
-        <v>3.05</v>
+        <v>3.55</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>1.0001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>3.55</v>
+        <v>5.05</v>
       </c>
       <c r="B8" t="n">
-        <v>1.3455</v>
+        <v>1.109</v>
       </c>
       <c r="C8" t="n">
         <v>3.55</v>
@@ -6783,18 +6810,18 @@
         <v>1.0095</v>
       </c>
       <c r="G8" t="n">
-        <v>3.55</v>
+        <v>4.07</v>
       </c>
       <c r="H8" t="n">
-        <v>1.0001</v>
+        <v>1.3203</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>4.05</v>
+        <v>5.55</v>
       </c>
       <c r="B9" t="n">
-        <v>1.2272</v>
+        <v>1.1065</v>
       </c>
       <c r="C9" t="n">
         <v>4.05</v>
@@ -6809,18 +6836,18 @@
         <v>1.432</v>
       </c>
       <c r="G9" t="n">
-        <v>4.07</v>
+        <v>4.57</v>
       </c>
       <c r="H9" t="n">
-        <v>1.3203</v>
+        <v>1.1731</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>4.55</v>
+        <v>6.07</v>
       </c>
       <c r="B10" t="n">
-        <v>1.1073</v>
+        <v>1.1074</v>
       </c>
       <c r="C10" t="n">
         <v>4.57</v>
@@ -6835,18 +6862,18 @@
         <v>1.1304</v>
       </c>
       <c r="G10" t="n">
-        <v>4.57</v>
+        <v>5.07</v>
       </c>
       <c r="H10" t="n">
-        <v>1.1731</v>
+        <v>1.1714</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5.05</v>
+        <v>6.57</v>
       </c>
       <c r="B11" t="n">
-        <v>1.109</v>
+        <v>1.1073</v>
       </c>
       <c r="C11" t="n">
         <v>5.07</v>
@@ -6861,18 +6888,18 @@
         <v>1.1325</v>
       </c>
       <c r="G11" t="n">
-        <v>5.07</v>
+        <v>5.57</v>
       </c>
       <c r="H11" t="n">
-        <v>1.1714</v>
+        <v>1.1696</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>5.55</v>
+        <v>7.07</v>
       </c>
       <c r="B12" t="n">
-        <v>1.1065</v>
+        <v>1.1069</v>
       </c>
       <c r="C12" t="n">
         <v>5.57</v>
@@ -6887,18 +6914,18 @@
         <v>1.1301</v>
       </c>
       <c r="G12" t="n">
-        <v>5.57</v>
+        <v>6.07</v>
       </c>
       <c r="H12" t="n">
-        <v>1.1696</v>
+        <v>1.1705</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>6.07</v>
+        <v>7.57</v>
       </c>
       <c r="B13" t="n">
-        <v>1.1074</v>
+        <v>1.1067</v>
       </c>
       <c r="C13" t="n">
         <v>6.07</v>
@@ -6913,18 +6940,18 @@
         <v>1.1302</v>
       </c>
       <c r="G13" t="n">
-        <v>6.07</v>
+        <v>6.57</v>
       </c>
       <c r="H13" t="n">
-        <v>1.1705</v>
+        <v>1.1701</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>6.57</v>
+        <v>8.07</v>
       </c>
       <c r="B14" t="n">
-        <v>1.1073</v>
+        <v>1.1079</v>
       </c>
       <c r="C14" t="n">
         <v>6.57</v>
@@ -6939,18 +6966,18 @@
         <v>1.1299</v>
       </c>
       <c r="G14" t="n">
-        <v>6.57</v>
+        <v>7.07</v>
       </c>
       <c r="H14" t="n">
-        <v>1.1701</v>
+        <v>1.1705</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>7.07</v>
+        <v>8.57</v>
       </c>
       <c r="B15" t="n">
-        <v>1.1069</v>
+        <v>1.107</v>
       </c>
       <c r="C15" t="n">
         <v>7.07</v>
@@ -6965,18 +6992,18 @@
         <v>1.1304</v>
       </c>
       <c r="G15" t="n">
-        <v>7.07</v>
+        <v>7.58</v>
       </c>
       <c r="H15" t="n">
-        <v>1.1705</v>
+        <v>1.1674</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>7.57</v>
+        <v>9.07</v>
       </c>
       <c r="B16" t="n">
-        <v>1.1067</v>
+        <v>1.1073</v>
       </c>
       <c r="C16" t="n">
         <v>7.57</v>
@@ -6991,18 +7018,18 @@
         <v>1.1298</v>
       </c>
       <c r="G16" t="n">
-        <v>7.58</v>
+        <v>8.08</v>
       </c>
       <c r="H16" t="n">
-        <v>1.1674</v>
+        <v>1.1677</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>8.07</v>
+        <v>9.57</v>
       </c>
       <c r="B17" t="n">
-        <v>1.1079</v>
+        <v>1.1093</v>
       </c>
       <c r="C17" t="n">
         <v>8.07</v>
@@ -7017,18 +7044,18 @@
         <v>1.1305</v>
       </c>
       <c r="G17" t="n">
-        <v>8.08</v>
+        <v>8.58</v>
       </c>
       <c r="H17" t="n">
-        <v>1.1677</v>
+        <v>1.1692</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>8.57</v>
+        <v>10.07</v>
       </c>
       <c r="B18" t="n">
-        <v>1.107</v>
+        <v>1.1008</v>
       </c>
       <c r="C18" t="n">
         <v>8.57</v>
@@ -7043,18 +7070,18 @@
         <v>1.1295</v>
       </c>
       <c r="G18" t="n">
-        <v>8.58</v>
+        <v>9.08</v>
       </c>
       <c r="H18" t="n">
-        <v>1.1692</v>
+        <v>1.1669</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>9.07</v>
+        <v>10.57</v>
       </c>
       <c r="B19" t="n">
-        <v>1.1073</v>
+        <v>1.1066</v>
       </c>
       <c r="C19" t="n">
         <v>9.07</v>
@@ -7069,18 +7096,18 @@
         <v>1.1292</v>
       </c>
       <c r="G19" t="n">
-        <v>9.08</v>
+        <v>9.58</v>
       </c>
       <c r="H19" t="n">
-        <v>1.1669</v>
+        <v>1.1695</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>9.57</v>
+        <v>11.07</v>
       </c>
       <c r="B20" t="n">
-        <v>1.1093</v>
+        <v>1.0994</v>
       </c>
       <c r="C20" t="n">
         <v>9.57</v>
@@ -7095,18 +7122,18 @@
         <v>1.1267</v>
       </c>
       <c r="G20" t="n">
-        <v>9.58</v>
+        <v>10.08</v>
       </c>
       <c r="H20" t="n">
-        <v>1.1695</v>
+        <v>1.1696</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>10.07</v>
+        <v>11.57</v>
       </c>
       <c r="B21" t="n">
-        <v>1.1008</v>
+        <v>1.1001</v>
       </c>
       <c r="C21" t="n">
         <v>10.07</v>
@@ -7121,18 +7148,18 @@
         <v>1.1288</v>
       </c>
       <c r="G21" t="n">
-        <v>10.08</v>
+        <v>10.58</v>
       </c>
       <c r="H21" t="n">
-        <v>1.1696</v>
+        <v>1.1717</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>10.57</v>
+        <v>12.07</v>
       </c>
       <c r="B22" t="n">
-        <v>1.1066</v>
+        <v>1.0991</v>
       </c>
       <c r="C22" t="n">
         <v>10.57</v>
@@ -7147,18 +7174,18 @@
         <v>1.1284</v>
       </c>
       <c r="G22" t="n">
-        <v>10.58</v>
+        <v>11.08</v>
       </c>
       <c r="H22" t="n">
-        <v>1.1717</v>
+        <v>1.1706</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>11.07</v>
+        <v>12.57</v>
       </c>
       <c r="B23" t="n">
-        <v>1.0994</v>
+        <v>1.101</v>
       </c>
       <c r="C23" t="n">
         <v>11.07</v>
@@ -7173,18 +7200,18 @@
         <v>1.1297</v>
       </c>
       <c r="G23" t="n">
-        <v>11.08</v>
+        <v>11.58</v>
       </c>
       <c r="H23" t="n">
-        <v>1.1706</v>
+        <v>1.1699</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>11.57</v>
+        <v>13.07</v>
       </c>
       <c r="B24" t="n">
-        <v>1.1001</v>
+        <v>1.1003</v>
       </c>
       <c r="C24" t="n">
         <v>11.57</v>
@@ -7199,18 +7226,18 @@
         <v>1.1286</v>
       </c>
       <c r="G24" t="n">
-        <v>11.58</v>
+        <v>12.08</v>
       </c>
       <c r="H24" t="n">
-        <v>1.1699</v>
+        <v>1.1664</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>12.07</v>
+        <v>13.57</v>
       </c>
       <c r="B25" t="n">
-        <v>1.0991</v>
+        <v>1.1001</v>
       </c>
       <c r="C25" t="n">
         <v>12.07</v>
@@ -7225,18 +7252,18 @@
         <v>1.1267</v>
       </c>
       <c r="G25" t="n">
-        <v>12.08</v>
+        <v>12.58</v>
       </c>
       <c r="H25" t="n">
-        <v>1.1664</v>
+        <v>1.1644</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>12.57</v>
+        <v>14.07</v>
       </c>
       <c r="B26" t="n">
-        <v>1.101</v>
+        <v>1.1027</v>
       </c>
       <c r="C26" t="n">
         <v>12.58</v>
@@ -7251,18 +7278,18 @@
         <v>1.1299</v>
       </c>
       <c r="G26" t="n">
-        <v>12.58</v>
+        <v>13.08</v>
       </c>
       <c r="H26" t="n">
-        <v>1.1644</v>
+        <v>1.1627</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>13.07</v>
+        <v>14.57</v>
       </c>
       <c r="B27" t="n">
-        <v>1.1003</v>
+        <v>1.1029</v>
       </c>
       <c r="C27" t="n">
         <v>13.08</v>
@@ -7277,18 +7304,18 @@
         <v>1.129</v>
       </c>
       <c r="G27" t="n">
-        <v>13.08</v>
+        <v>13.58</v>
       </c>
       <c r="H27" t="n">
-        <v>1.1627</v>
+        <v>1.1641</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>13.57</v>
+        <v>15.07</v>
       </c>
       <c r="B28" t="n">
-        <v>1.1001</v>
+        <v>1.0996</v>
       </c>
       <c r="C28" t="n">
         <v>13.58</v>
@@ -7303,18 +7330,18 @@
         <v>1.1283</v>
       </c>
       <c r="G28" t="n">
-        <v>13.58</v>
+        <v>14.08</v>
       </c>
       <c r="H28" t="n">
-        <v>1.1641</v>
+        <v>1.1651</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>14.07</v>
+        <v>15.57</v>
       </c>
       <c r="B29" t="n">
-        <v>1.1027</v>
+        <v>1.0996</v>
       </c>
       <c r="C29" t="n">
         <v>14.08</v>
@@ -7329,18 +7356,18 @@
         <v>1.1287</v>
       </c>
       <c r="G29" t="n">
-        <v>14.08</v>
+        <v>14.58</v>
       </c>
       <c r="H29" t="n">
-        <v>1.1651</v>
+        <v>1.1625</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>14.57</v>
+        <v>16.07</v>
       </c>
       <c r="B30" t="n">
-        <v>1.1029</v>
+        <v>1.0991</v>
       </c>
       <c r="C30" t="n">
         <v>14.58</v>
@@ -7355,18 +7382,18 @@
         <v>1.1271</v>
       </c>
       <c r="G30" t="n">
-        <v>14.58</v>
+        <v>15.08</v>
       </c>
       <c r="H30" t="n">
-        <v>1.1625</v>
+        <v>1.1654</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>15.07</v>
+        <v>16.72</v>
       </c>
       <c r="B31" t="n">
-        <v>1.0996</v>
+        <v>1.1009</v>
       </c>
       <c r="C31" t="n">
         <v>15.08</v>
@@ -7381,18 +7408,18 @@
         <v>1.1281</v>
       </c>
       <c r="G31" t="n">
-        <v>15.08</v>
+        <v>15.58</v>
       </c>
       <c r="H31" t="n">
-        <v>1.1654</v>
+        <v>1.1636</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>15.57</v>
+        <v>17.25</v>
       </c>
       <c r="B32" t="n">
-        <v>1.0996</v>
+        <v>1.1024</v>
       </c>
       <c r="C32" t="n">
         <v>15.58</v>
@@ -7407,18 +7434,18 @@
         <v>1.1282</v>
       </c>
       <c r="G32" t="n">
-        <v>15.58</v>
+        <v>16.08</v>
       </c>
       <c r="H32" t="n">
-        <v>1.1636</v>
+        <v>1.162</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>16.07</v>
+        <v>17.78</v>
       </c>
       <c r="B33" t="n">
-        <v>1.0991</v>
+        <v>1.0995</v>
       </c>
       <c r="C33" t="n">
         <v>16.08</v>
@@ -7433,18 +7460,18 @@
         <v>1.1283</v>
       </c>
       <c r="G33" t="n">
-        <v>16.08</v>
+        <v>16.58</v>
       </c>
       <c r="H33" t="n">
-        <v>1.162</v>
+        <v>1.1636</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>16.72</v>
+        <v>18.28</v>
       </c>
       <c r="B34" t="n">
-        <v>1.1009</v>
+        <v>1.0995</v>
       </c>
       <c r="C34" t="n">
         <v>16.58</v>
@@ -7459,19 +7486,13 @@
         <v>1.129</v>
       </c>
       <c r="G34" t="n">
-        <v>16.58</v>
+        <v>17.08</v>
       </c>
       <c r="H34" t="n">
-        <v>1.1636</v>
+        <v>1.1637</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="n">
-        <v>17.25</v>
-      </c>
-      <c r="B35" t="n">
-        <v>1.1024</v>
-      </c>
       <c r="C35" t="n">
         <v>17.08</v>
       </c>
@@ -7485,19 +7506,13 @@
         <v>1.1289</v>
       </c>
       <c r="G35" t="n">
-        <v>17.08</v>
+        <v>17.6</v>
       </c>
       <c r="H35" t="n">
-        <v>1.1637</v>
+        <v>1.1677</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="n">
-        <v>17.78</v>
-      </c>
-      <c r="B36" t="n">
-        <v>1.0995</v>
-      </c>
       <c r="C36" t="n">
         <v>17.58</v>
       </c>
@@ -7511,19 +7526,13 @@
         <v>1.1279</v>
       </c>
       <c r="G36" t="n">
-        <v>17.6</v>
+        <v>18.12</v>
       </c>
       <c r="H36" t="n">
-        <v>1.1677</v>
+        <v>1.1627</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="n">
-        <v>18.28</v>
-      </c>
-      <c r="B37" t="n">
-        <v>1.0995</v>
-      </c>
       <c r="C37" t="n">
         <v>18.08</v>
       </c>
@@ -7537,10 +7546,10 @@
         <v>1.1286</v>
       </c>
       <c r="G37" t="n">
-        <v>18.12</v>
+        <v>18.63</v>
       </c>
       <c r="H37" t="n">
-        <v>1.1627</v>
+        <v>1.1603</v>
       </c>
     </row>
     <row r="38">
@@ -7555,12 +7564,6 @@
       </c>
       <c r="F38" t="n">
         <v>1.127</v>
-      </c>
-      <c r="G38" t="n">
-        <v>18.63</v>
-      </c>
-      <c r="H38" t="n">
-        <v>1.1603</v>
       </c>
     </row>
     <row r="39">

</xml_diff>

<commit_message>
fig14 xlsx: explicit scatterStyle=lineMarker and blanks=span so Excel draws continuous lines
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig14_lines.xlsx
+++ b/figs/data/fig14_lines.xlsx
@@ -148,6 +148,7 @@
     </title>
     <plotArea>
       <scatterChart>
+        <scatterStyle val="lineMarker"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -361,7 +362,7 @@
       <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
+    <dispBlanksAs val="span"/>
   </chart>
 </chartSpace>
 </file>
@@ -387,6 +388,7 @@
     </title>
     <plotArea>
       <scatterChart>
+        <scatterStyle val="lineMarker"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -600,7 +602,7 @@
       <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
+    <dispBlanksAs val="span"/>
   </chart>
 </chartSpace>
 </file>
@@ -626,6 +628,7 @@
     </title>
     <plotArea>
       <scatterChart>
+        <scatterStyle val="lineMarker"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -839,7 +842,7 @@
       <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
+    <dispBlanksAs val="span"/>
   </chart>
 </chartSpace>
 </file>
@@ -865,6 +868,7 @@
     </title>
     <plotArea>
       <scatterChart>
+        <scatterStyle val="lineMarker"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -1078,7 +1082,7 @@
       <legendPos val="b"/>
     </legend>
     <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
+    <dispBlanksAs val="span"/>
   </chart>
 </chartSpace>
 </file>

</xml_diff>

<commit_message>
Switch time shown: red labelled line in Fig.7/Fig.14 PNG and as a legend series in fig7.xlsx / fig14_lines.xlsx
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig14_lines.xlsx
+++ b/figs/data/fig14_lines.xlsx
@@ -293,6 +293,41 @@
           </yVal>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'OLTP→Varmail'!L1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="E5484D"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'OLTP→Varmail'!$K$2:$K$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'OLTP→Varmail'!$L$2:$L$3</f>
+            </numRef>
+          </yVal>
+        </ser>
         <axId val="10"/>
         <axId val="20"/>
       </scatterChart>
@@ -532,6 +567,41 @@
             </numRef>
           </yVal>
           <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'FIO-Fast→Varmail'!L1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="E5484D"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'FIO-Fast→Varmail'!$K$2:$K$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'FIO-Fast→Varmail'!$L$2:$L$3</f>
+            </numRef>
+          </yVal>
         </ser>
         <axId val="10"/>
         <axId val="20"/>
@@ -773,6 +843,41 @@
           </yVal>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'YCSB-A→YCSB-B'!L1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="E5484D"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'YCSB-A→YCSB-B'!$K$2:$K$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'YCSB-A→YCSB-B'!$L$2:$L$3</f>
+            </numRef>
+          </yVal>
+        </ser>
         <axId val="10"/>
         <axId val="20"/>
       </scatterChart>
@@ -1013,6 +1118,41 @@
           </yVal>
           <smooth val="0"/>
         </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'YCSB-A→OLTP'!L1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="E5484D"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'YCSB-A→OLTP'!$K$2:$K$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'YCSB-A→OLTP'!$L$2:$L$3</f>
+            </numRef>
+          </yVal>
+        </ser>
         <axId val="10"/>
         <axId val="20"/>
       </scatterChart>
@@ -1091,7 +1231,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>11</col>
+      <col>13</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -1118,7 +1258,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>11</col>
+      <col>13</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -1145,7 +1285,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>11</col>
+      <col>13</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -1172,7 +1312,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>11</col>
+      <col>13</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -1484,7 +1624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="10" max="10"/>
@@ -1536,6 +1676,16 @@
           <t>워크로드 전환 시점(분)</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>전환 시간</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>워크로드 전환 (v4 기준 16.0분)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -1567,6 +1717,12 @@
           <t>iCAT-v4: 16.0</t>
         </is>
       </c>
+      <c r="K2" t="n">
+        <v>16.03</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1.12</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -1597,6 +1753,12 @@
         <is>
           <t>CAT-47 (최적): 15.6</t>
         </is>
+      </c>
+      <c r="K3" t="n">
+        <v>16.03</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="4">
@@ -3117,7 +3279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J90"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="10" max="10"/>
@@ -3169,6 +3331,16 @@
           <t>워크로드 전환 시점(분)</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>전환 시간</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>워크로드 전환 (v4 기준 30.0분)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -3200,6 +3372,12 @@
           <t>iCAT-v4: 30.0</t>
         </is>
       </c>
+      <c r="K2" t="n">
+        <v>30</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1.45</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -3230,6 +3408,12 @@
         <is>
           <t>CAT-47 (최적): 30.0</t>
         </is>
+      </c>
+      <c r="K3" t="n">
+        <v>30</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4.41</v>
       </c>
     </row>
     <row r="4">
@@ -5516,7 +5700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="10" max="10"/>
@@ -5568,6 +5752,16 @@
           <t>워크로드 전환 시점(분)</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>전환 시간</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>워크로드 전환 (v4 기준 15.8분)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -5599,6 +5793,12 @@
           <t>iCAT-v4: 15.8</t>
         </is>
       </c>
+      <c r="K2" t="n">
+        <v>15.77</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1.25</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -5629,6 +5829,12 @@
         <is>
           <t>CAT-47 (최적): 16.9</t>
         </is>
+      </c>
+      <c r="K3" t="n">
+        <v>15.77</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1.7</v>
       </c>
     </row>
     <row r="4">
@@ -6565,7 +6771,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="10" max="10"/>
@@ -6617,6 +6823,16 @@
           <t>워크로드 전환 시점(분)</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>전환 시간</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>워크로드 전환 (v4 기준 3.5분)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -6648,6 +6864,12 @@
           <t>iCAT-v4: 3.5</t>
         </is>
       </c>
+      <c r="K2" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.92</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -6678,6 +6900,12 @@
         <is>
           <t>CAT-47 (최적): 4.0</t>
         </is>
+      </c>
+      <c r="K3" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2.04</v>
       </c>
     </row>
     <row r="4">

</xml_diff>